<commit_message>
refactor(epirank): store trajectory as (space, iteration) and fix indexing
- transpose trajectory to (N, T) so row index = space unit, column index = iteration; update all accesses in compute_epidemic_risk, M1 log formatter and M1 transient plots
- refresh ERA results for 改 (305/306 loops) and 改_Germany (310 loops)
</commit_message>
<xml_diff>
--- a/EpiRank_改/ERA_result_reverse_seqday_d_0.95_loops_306.xlsx
+++ b/EpiRank_改/ERA_result_reverse_seqday_d_0.95_loops_306.xlsx
@@ -714,10 +714,10 @@
         <v>0.012835</v>
       </c>
       <c r="Y2" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z2" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA2" s="3" t="n">
         <v>9</v>
@@ -1024,10 +1024,10 @@
         <v>0.012838</v>
       </c>
       <c r="Y4" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z4" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA4" s="3" t="n">
         <v>11</v>
@@ -1179,10 +1179,10 @@
         <v>0.01205</v>
       </c>
       <c r="Y5" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z5" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA5" s="3" t="n">
         <v>11</v>
@@ -1334,10 +1334,10 @@
         <v>0.006652</v>
       </c>
       <c r="Y6" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z6" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA6" s="3" t="n">
         <v>11</v>
@@ -1636,10 +1636,10 @@
         <v>0.016941</v>
       </c>
       <c r="Y8" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z8" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA8" s="3" t="n">
         <v>8</v>
@@ -1938,10 +1938,10 @@
         <v>0.011997</v>
       </c>
       <c r="Y10" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z10" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA10" s="3" t="n">
         <v>4</v>
@@ -3138,10 +3138,10 @@
         <v>0.004698</v>
       </c>
       <c r="Y18" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z18" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA18" s="3" t="n">
         <v>4</v>
@@ -3688,10 +3688,10 @@
         <v>0.009729</v>
       </c>
       <c r="Y22" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z22" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA22" s="3" t="n">
         <v>24</v>
@@ -3948,7 +3948,7 @@
         <v>0.007023</v>
       </c>
       <c r="Y24" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z24" s="3" t="n">
         <v>-0</v>
@@ -4598,7 +4598,7 @@
         <v>0.004713</v>
       </c>
       <c r="Y29" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z29" s="3" t="n">
         <v>0</v>
@@ -4988,7 +4988,7 @@
         <v>0.008265</v>
       </c>
       <c r="Y32" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z32" s="3" t="n">
         <v>0</v>
@@ -5118,10 +5118,10 @@
         <v>0.005408</v>
       </c>
       <c r="Y33" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z33" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA33" s="3" t="n">
         <v>7</v>
@@ -5478,10 +5478,10 @@
         <v>0.01038</v>
       </c>
       <c r="Y36" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z36" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA36" s="3" t="n">
         <v>0</v>
@@ -6321,7 +6321,7 @@
         <v>0</v>
       </c>
       <c r="Z43" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA43" s="3" t="n">
         <v>2</v>
@@ -6438,10 +6438,10 @@
         <v>0.007706</v>
       </c>
       <c r="Y44" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z44" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA44" s="3" t="n">
         <v>2</v>
@@ -6558,10 +6558,10 @@
         <v>0.006149</v>
       </c>
       <c r="Y45" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z45" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA45" s="3" t="n">
         <v>5</v>
@@ -6798,10 +6798,10 @@
         <v>0.005831</v>
       </c>
       <c r="Y47" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z47" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA47" s="3" t="n">
         <v>0</v>
@@ -6918,10 +6918,10 @@
         <v>0.006948</v>
       </c>
       <c r="Y48" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z48" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA48" s="3" t="n">
         <v>3</v>
@@ -7518,7 +7518,7 @@
         <v>0.005555</v>
       </c>
       <c r="Y53" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z53" s="3" t="n">
         <v>0</v>
@@ -7878,10 +7878,10 @@
         <v>0.004587</v>
       </c>
       <c r="Y56" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z56" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA56" s="3" t="n">
         <v>2</v>
@@ -8598,10 +8598,10 @@
         <v>0.006096</v>
       </c>
       <c r="Y62" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z62" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA62" s="3" t="n">
         <v>1</v>
@@ -8958,10 +8958,10 @@
         <v>0.004618</v>
       </c>
       <c r="Y65" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z65" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA65" s="3" t="n">
         <v>6</v>
@@ -9198,7 +9198,7 @@
         <v>0.0015</v>
       </c>
       <c r="Y67" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z67" s="3" t="n">
         <v>-0</v>
@@ -9548,7 +9548,7 @@
         <v>0.002648</v>
       </c>
       <c r="Y70" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z70" s="3" t="n">
         <v>-0</v>
@@ -9878,10 +9878,10 @@
         <v>0.003248</v>
       </c>
       <c r="Y73" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z73" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA73" s="3" t="n">
         <v>3</v>
@@ -10978,7 +10978,7 @@
         <v>0.002498</v>
       </c>
       <c r="Y83" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z83" s="3" t="n">
         <v>-0</v>
@@ -11198,10 +11198,10 @@
         <v>0.003041</v>
       </c>
       <c r="Y85" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z85" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA85" s="3" t="n">
         <v>1</v>
@@ -11531,7 +11531,7 @@
         <v>0</v>
       </c>
       <c r="Z88" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA88" s="3" t="n">
         <v>2</v>
@@ -11858,10 +11858,10 @@
         <v>0.002947</v>
       </c>
       <c r="Y91" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z91" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA91" s="3" t="n">
         <v>3</v>
@@ -11971,7 +11971,7 @@
         <v>0</v>
       </c>
       <c r="Z92" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA92" s="3" t="n">
         <v>1</v>
@@ -12628,10 +12628,10 @@
         <v>0.003197</v>
       </c>
       <c r="Y98" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z98" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA98" s="3" t="n">
         <v>1</v>
@@ -13178,10 +13178,10 @@
         <v>0.003781</v>
       </c>
       <c r="Y103" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z103" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA103" s="3" t="n">
         <v>0</v>
@@ -14058,10 +14058,10 @@
         <v>0.003672</v>
       </c>
       <c r="Y111" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z111" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA111" s="3" t="n">
         <v>0</v>
@@ -14278,7 +14278,7 @@
         <v>0.002715</v>
       </c>
       <c r="Y113" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z113" s="3" t="n">
         <v>0</v>
@@ -14498,10 +14498,10 @@
         <v>0.002806</v>
       </c>
       <c r="Y115" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z115" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA115" s="3" t="n">
         <v>0</v>
@@ -14608,7 +14608,7 @@
         <v>0.005244</v>
       </c>
       <c r="Y116" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z116" s="3" t="n">
         <v>0</v>
@@ -14718,10 +14718,10 @@
         <v>0.004473</v>
       </c>
       <c r="Y117" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z117" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA117" s="3" t="n">
         <v>1</v>
@@ -15268,10 +15268,10 @@
         <v>0.002014</v>
       </c>
       <c r="Y122" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z122" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA122" s="3" t="n">
         <v>3</v>
@@ -15491,7 +15491,7 @@
         <v>-0</v>
       </c>
       <c r="Z124" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA124" s="3" t="n">
         <v>3</v>
@@ -16148,10 +16148,10 @@
         <v>0.002496</v>
       </c>
       <c r="Y130" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z130" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA130" s="3" t="n">
         <v>1</v>
@@ -16808,10 +16808,10 @@
         <v>0.002381</v>
       </c>
       <c r="Y136" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z136" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA136" s="3" t="n">
         <v>2</v>
@@ -17138,7 +17138,7 @@
         <v>0.001759</v>
       </c>
       <c r="Y139" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z139" s="3" t="n">
         <v>-0</v>
@@ -17248,10 +17248,10 @@
         <v>0.002964</v>
       </c>
       <c r="Y140" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z140" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA140" s="3" t="n">
         <v>3</v>
@@ -17358,7 +17358,7 @@
         <v>0.00302</v>
       </c>
       <c r="Y141" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z141" s="3" t="n">
         <v>-0</v>
@@ -17468,10 +17468,10 @@
         <v>0.001286</v>
       </c>
       <c r="Y142" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z142" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA142" s="3" t="n">
         <v>1</v>
@@ -18458,10 +18458,10 @@
         <v>0.00181</v>
       </c>
       <c r="Y151" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z151" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA151" s="3" t="n">
         <v>1</v>
@@ -18898,10 +18898,10 @@
         <v>0.002578</v>
       </c>
       <c r="Y155" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z155" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA155" s="3" t="n">
         <v>0</v>
@@ -19118,10 +19118,10 @@
         <v>0.001714</v>
       </c>
       <c r="Y157" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z157" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA157" s="3" t="n">
         <v>2</v>
@@ -19228,10 +19228,10 @@
         <v>0.002491</v>
       </c>
       <c r="Y158" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z158" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA158" s="3" t="n">
         <v>2</v>
@@ -19338,7 +19338,7 @@
         <v>0.002147</v>
       </c>
       <c r="Y159" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z159" s="3" t="n">
         <v>0</v>
@@ -19668,7 +19668,7 @@
         <v>0.003364</v>
       </c>
       <c r="Y162" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z162" s="3" t="n">
         <v>-0</v>
@@ -19778,7 +19778,7 @@
         <v>0.002174</v>
       </c>
       <c r="Y163" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z163" s="3" t="n">
         <v>-0</v>
@@ -20438,10 +20438,10 @@
         <v>0.001295</v>
       </c>
       <c r="Y169" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z169" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA169" s="3" t="n">
         <v>0</v>
@@ -20658,10 +20658,10 @@
         <v>0.001901</v>
       </c>
       <c r="Y171" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z171" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA171" s="3" t="n">
         <v>0</v>
@@ -20878,10 +20878,10 @@
         <v>0.001797</v>
       </c>
       <c r="Y173" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z173" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA173" s="3" t="n">
         <v>0</v>
@@ -21098,10 +21098,10 @@
         <v>0.001399</v>
       </c>
       <c r="Y175" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z175" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA175" s="3" t="n">
         <v>1</v>
@@ -21208,10 +21208,10 @@
         <v>0.002542</v>
       </c>
       <c r="Y176" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z176" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA176" s="3" t="n">
         <v>1</v>
@@ -21318,10 +21318,10 @@
         <v>0.001307</v>
       </c>
       <c r="Y177" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z177" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA177" s="3" t="n">
         <v>0</v>
@@ -21428,7 +21428,7 @@
         <v>0.002004</v>
       </c>
       <c r="Y178" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z178" s="3" t="n">
         <v>0</v>
@@ -21758,10 +21758,10 @@
         <v>0.002618</v>
       </c>
       <c r="Y181" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z181" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA181" s="3" t="n">
         <v>0</v>
@@ -21871,7 +21871,7 @@
         <v>0</v>
       </c>
       <c r="Z182" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA182" s="3" t="n">
         <v>1</v>
@@ -22418,10 +22418,10 @@
         <v>0.002818</v>
       </c>
       <c r="Y187" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z187" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA187" s="3" t="n">
         <v>0</v>
@@ -22641,7 +22641,7 @@
         <v>0</v>
       </c>
       <c r="Z189" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA189" s="3" t="n">
         <v>1</v>
@@ -22748,10 +22748,10 @@
         <v>0.002087</v>
       </c>
       <c r="Y190" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z190" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA190" s="3" t="n">
         <v>0</v>
@@ -23191,7 +23191,7 @@
         <v>0</v>
       </c>
       <c r="Z194" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA194" s="3" t="n">
         <v>0</v>
@@ -23298,7 +23298,7 @@
         <v>0.001708</v>
       </c>
       <c r="Y195" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z195" s="3" t="n">
         <v>-0</v>
@@ -23628,10 +23628,10 @@
         <v>0.001192</v>
       </c>
       <c r="Y198" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z198" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA198" s="3" t="n">
         <v>0</v>
@@ -23848,10 +23848,10 @@
         <v>0.001259</v>
       </c>
       <c r="Y200" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z200" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA200" s="3" t="n">
         <v>1</v>
@@ -24068,10 +24068,10 @@
         <v>0.001326</v>
       </c>
       <c r="Y202" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z202" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA202" s="3" t="n">
         <v>0</v>
@@ -24398,7 +24398,7 @@
         <v>0.001495</v>
       </c>
       <c r="Y205" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z205" s="3" t="n">
         <v>0</v>
@@ -24511,7 +24511,7 @@
         <v>0</v>
       </c>
       <c r="Z206" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA206" s="3" t="n">
         <v>3</v>
@@ -24838,10 +24838,10 @@
         <v>0.001782</v>
       </c>
       <c r="Y209" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z209" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA209" s="3" t="n">
         <v>2</v>
@@ -24948,10 +24948,10 @@
         <v>0.002238</v>
       </c>
       <c r="Y210" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z210" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA210" s="3" t="n">
         <v>0</v>
@@ -25168,10 +25168,10 @@
         <v>0.002084</v>
       </c>
       <c r="Y212" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z212" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA212" s="3" t="n">
         <v>2</v>
@@ -25388,10 +25388,10 @@
         <v>0.001245</v>
       </c>
       <c r="Y214" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z214" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA214" s="3" t="n">
         <v>0</v>
@@ -25501,7 +25501,7 @@
         <v>0</v>
       </c>
       <c r="Z215" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA215" s="3" t="n">
         <v>1</v>
@@ -25608,7 +25608,7 @@
         <v>0.001081</v>
       </c>
       <c r="Y216" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z216" s="3" t="n">
         <v>-0</v>
@@ -25938,7 +25938,7 @@
         <v>0.00315</v>
       </c>
       <c r="Y219" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z219" s="3" t="n">
         <v>-0</v>
@@ -26488,10 +26488,10 @@
         <v>0.00209</v>
       </c>
       <c r="Y224" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z224" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA224" s="3" t="n">
         <v>1</v>
@@ -26691,7 +26691,7 @@
         <v>0</v>
       </c>
       <c r="Z226" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA226" s="3" t="n">
         <v>1</v>
@@ -26888,10 +26888,10 @@
         <v>0.00125</v>
       </c>
       <c r="Y228" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z228" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA228" s="3" t="n">
         <v>0</v>
@@ -26988,7 +26988,7 @@
         <v>0.00135</v>
       </c>
       <c r="Y229" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z229" s="3" t="n">
         <v>-0</v>
@@ -27088,10 +27088,10 @@
         <v>0.001999</v>
       </c>
       <c r="Y230" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z230" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA230" s="3" t="n">
         <v>0</v>
@@ -27188,10 +27188,10 @@
         <v>0.001237</v>
       </c>
       <c r="Y231" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z231" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA231" s="3" t="n">
         <v>5</v>
@@ -27391,7 +27391,7 @@
         <v>-0</v>
       </c>
       <c r="Z233" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA233" s="3" t="n">
         <v>0</v>
@@ -27688,7 +27688,7 @@
         <v>0.0008140000000000001</v>
       </c>
       <c r="Y236" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z236" s="3" t="n">
         <v>-0</v>
@@ -27791,7 +27791,7 @@
         <v>0</v>
       </c>
       <c r="Z237" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA237" s="3" t="n">
         <v>2</v>
@@ -27888,7 +27888,7 @@
         <v>0.001309</v>
       </c>
       <c r="Y238" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z238" s="3" t="n">
         <v>0</v>
@@ -28088,7 +28088,7 @@
         <v>0.001577</v>
       </c>
       <c r="Y240" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z240" s="3" t="n">
         <v>0</v>
@@ -28188,10 +28188,10 @@
         <v>0.001152</v>
       </c>
       <c r="Y241" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z241" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA241" s="3" t="n">
         <v>0</v>
@@ -28288,10 +28288,10 @@
         <v>0.001386</v>
       </c>
       <c r="Y242" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z242" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA242" s="3" t="n">
         <v>0</v>
@@ -28388,7 +28388,7 @@
         <v>0.001556</v>
       </c>
       <c r="Y243" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z243" s="3" t="n">
         <v>-0</v>
@@ -28491,7 +28491,7 @@
         <v>-0</v>
       </c>
       <c r="Z244" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA244" s="3" t="n">
         <v>1</v>
@@ -28888,10 +28888,10 @@
         <v>0.000905</v>
       </c>
       <c r="Y248" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z248" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA248" s="3" t="n">
         <v>0</v>
@@ -29288,7 +29288,7 @@
         <v>0.001248</v>
       </c>
       <c r="Y252" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z252" s="3" t="n">
         <v>0</v>
@@ -29388,10 +29388,10 @@
         <v>0.00164</v>
       </c>
       <c r="Y253" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z253" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA253" s="3" t="n">
         <v>0</v>
@@ -29491,7 +29491,7 @@
         <v>0</v>
       </c>
       <c r="Z254" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA254" s="3" t="n">
         <v>3</v>
@@ -29588,10 +29588,10 @@
         <v>0.000995</v>
       </c>
       <c r="Y255" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z255" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA255" s="3" t="n">
         <v>0</v>
@@ -29788,7 +29788,7 @@
         <v>0.001036</v>
       </c>
       <c r="Y257" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z257" s="3" t="n">
         <v>-0</v>
@@ -30388,10 +30388,10 @@
         <v>0.001296</v>
       </c>
       <c r="Y263" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z263" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA263" s="3" t="n">
         <v>1</v>
@@ -30888,10 +30888,10 @@
         <v>0.00079</v>
       </c>
       <c r="Y268" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z268" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA268" s="3" t="n">
         <v>1</v>
@@ -30988,7 +30988,7 @@
         <v>0.001019</v>
       </c>
       <c r="Y269" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z269" s="3" t="n">
         <v>-0</v>
@@ -31088,10 +31088,10 @@
         <v>0.001378</v>
       </c>
       <c r="Y270" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z270" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA270" s="3" t="n">
         <v>2</v>
@@ -31188,7 +31188,7 @@
         <v>0.001352</v>
       </c>
       <c r="Y271" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z271" s="3" t="n">
         <v>0</v>
@@ -31388,7 +31388,7 @@
         <v>0.001118</v>
       </c>
       <c r="Y273" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z273" s="3" t="n">
         <v>0</v>
@@ -31591,7 +31591,7 @@
         <v>0</v>
       </c>
       <c r="Z275" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA275" s="3" t="n">
         <v>0</v>
@@ -31688,10 +31688,10 @@
         <v>0.001773</v>
       </c>
       <c r="Y276" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z276" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA276" s="3" t="n">
         <v>1</v>
@@ -31788,7 +31788,7 @@
         <v>0.000672</v>
       </c>
       <c r="Y277" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z277" s="3" t="n">
         <v>-0</v>
@@ -31888,10 +31888,10 @@
         <v>0.000785</v>
       </c>
       <c r="Y278" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z278" s="3" t="n">
         <v>-0</v>
-      </c>
-      <c r="Z278" s="3" t="n">
-        <v>0</v>
       </c>
       <c r="AA278" s="3" t="n">
         <v>0</v>
@@ -32388,7 +32388,7 @@
         <v>0.00126</v>
       </c>
       <c r="Y283" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z283" s="3" t="n">
         <v>-0</v>
@@ -32488,10 +32488,10 @@
         <v>0.001506</v>
       </c>
       <c r="Y284" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z284" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA284" s="3" t="n">
         <v>2</v>
@@ -32588,10 +32588,10 @@
         <v>0.00134</v>
       </c>
       <c r="Y285" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z285" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA285" s="3" t="n">
         <v>0</v>
@@ -32688,10 +32688,10 @@
         <v>0.000804</v>
       </c>
       <c r="Y286" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z286" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA286" s="3" t="n">
         <v>1</v>
@@ -33088,7 +33088,7 @@
         <v>0.000883</v>
       </c>
       <c r="Y290" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z290" s="3" t="n">
         <v>0</v>
@@ -33288,10 +33288,10 @@
         <v>0.00087</v>
       </c>
       <c r="Y292" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z292" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA292" s="3" t="n">
         <v>1</v>
@@ -33488,10 +33488,10 @@
         <v>0.0009479999999999999</v>
       </c>
       <c r="Y294" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z294" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA294" s="3" t="n">
         <v>0</v>
@@ -33688,7 +33688,7 @@
         <v>0.001087</v>
       </c>
       <c r="Y296" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z296" s="3" t="n">
         <v>-0</v>
@@ -33791,7 +33791,7 @@
         <v>-0</v>
       </c>
       <c r="Z297" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA297" s="3" t="n">
         <v>0</v>
@@ -33888,10 +33888,10 @@
         <v>0.00108</v>
       </c>
       <c r="Y298" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z298" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA298" s="3" t="n">
         <v>2</v>
@@ -34191,7 +34191,7 @@
         <v>0</v>
       </c>
       <c r="Z301" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA301" s="3" t="n">
         <v>1</v>
@@ -34291,7 +34291,7 @@
         <v>0</v>
       </c>
       <c r="Z302" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA302" s="3" t="n">
         <v>0</v>
@@ -34388,7 +34388,7 @@
         <v>0.001097</v>
       </c>
       <c r="Y303" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z303" s="3" t="n">
         <v>0</v>
@@ -34488,10 +34488,10 @@
         <v>0.000908</v>
       </c>
       <c r="Y304" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z304" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA304" s="3" t="n">
         <v>0</v>
@@ -34688,7 +34688,7 @@
         <v>0.000803</v>
       </c>
       <c r="Y306" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z306" s="3" t="n">
         <v>-0</v>
@@ -34888,10 +34888,10 @@
         <v>0.001184</v>
       </c>
       <c r="Y308" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z308" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA308" s="3" t="n">
         <v>0</v>
@@ -35188,7 +35188,7 @@
         <v>0.000919</v>
       </c>
       <c r="Y311" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z311" s="3" t="n">
         <v>-0</v>
@@ -35288,10 +35288,10 @@
         <v>0.000773</v>
       </c>
       <c r="Y312" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z312" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA312" s="3" t="n">
         <v>0</v>
@@ -35488,7 +35488,7 @@
         <v>0.000827</v>
       </c>
       <c r="Y314" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z314" s="3" t="n">
         <v>0</v>
@@ -35688,7 +35688,7 @@
         <v>0.000803</v>
       </c>
       <c r="Y316" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z316" s="3" t="n">
         <v>0</v>
@@ -35991,7 +35991,7 @@
         <v>0</v>
       </c>
       <c r="Z319" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA319" s="3" t="n">
         <v>0</v>
@@ -36588,10 +36588,10 @@
         <v>0.000819</v>
       </c>
       <c r="Y325" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z325" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA325" s="3" t="n">
         <v>3</v>
@@ -36888,10 +36888,10 @@
         <v>0.001202</v>
       </c>
       <c r="Y328" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z328" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA328" s="3" t="n">
         <v>0</v>
@@ -36988,10 +36988,10 @@
         <v>0.00122</v>
       </c>
       <c r="Y329" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z329" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA329" s="3" t="n">
         <v>0</v>
@@ -37588,7 +37588,7 @@
         <v>0.000763</v>
       </c>
       <c r="Y335" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z335" s="3" t="n">
         <v>0</v>
@@ -37688,7 +37688,7 @@
         <v>0.001203</v>
       </c>
       <c r="Y336" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z336" s="3" t="n">
         <v>-0</v>
@@ -38288,10 +38288,10 @@
         <v>0.000725</v>
       </c>
       <c r="Y342" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z342" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA342" s="3" t="n">
         <v>1</v>
@@ -38588,7 +38588,7 @@
         <v>0.000561</v>
       </c>
       <c r="Y345" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z345" s="3" t="n">
         <v>-0</v>
@@ -38788,10 +38788,10 @@
         <v>0.000592</v>
       </c>
       <c r="Y347" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z347" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA347" s="3" t="n">
         <v>0</v>
@@ -39288,10 +39288,10 @@
         <v>0.000518</v>
       </c>
       <c r="Y352" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z352" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA352" s="3" t="n">
         <v>0</v>
@@ -39564,10 +39564,10 @@
         <v>0.529801</v>
       </c>
       <c r="Y356" s="3" t="n">
-        <v>0.108565</v>
+        <v>0.118288</v>
       </c>
       <c r="Z356" s="3" t="n">
-        <v>0.080931</v>
+        <v>0.122572</v>
       </c>
       <c r="AB356" s="3" t="n">
         <v>0.635544</v>
@@ -39626,10 +39626,10 @@
         <v>0.445424</v>
       </c>
       <c r="Y358" s="3" t="n">
-        <v>0.423203</v>
+        <v>0.329352</v>
       </c>
       <c r="Z358" s="3" t="n">
-        <v>0.390298</v>
+        <v>0.359123</v>
       </c>
       <c r="AA358" s="3" t="n">
         <v>0.551809</v>
@@ -40001,10 +40001,10 @@
         <v>0.386474</v>
       </c>
       <c r="D8" t="n">
-        <v>0.423203</v>
+        <v>0.329352</v>
       </c>
       <c r="E8" t="n">
-        <v>0.31968</v>
+        <v>0.253445</v>
       </c>
       <c r="F8" t="n">
         <v>0.2988505747126437</v>
@@ -40031,10 +40031,10 @@
         <v>0.216528</v>
       </c>
       <c r="D9" t="n">
-        <v>0.108565</v>
+        <v>0.118288</v>
       </c>
       <c r="E9" t="n">
-        <v>0.081109</v>
+        <v>0.09131400000000001</v>
       </c>
       <c r="F9" t="n">
         <v>0.1641791044776119</v>
@@ -40061,10 +40061,10 @@
         <v>0.41859</v>
       </c>
       <c r="D10" t="n">
-        <v>0.373811</v>
+        <v>0.282654</v>
       </c>
       <c r="E10" t="n">
-        <v>0.303776</v>
+        <v>0.228</v>
       </c>
       <c r="F10" t="n">
         <v>0.3636363636363636</v>
@@ -40091,10 +40091,10 @@
         <v>0.397421</v>
       </c>
       <c r="D11" t="n">
-        <v>0.390298</v>
+        <v>0.359123</v>
       </c>
       <c r="E11" t="n">
-        <v>0.29368</v>
+        <v>0.274224</v>
       </c>
       <c r="F11" t="n">
         <v>0.3333333333333333</v>
@@ -40121,10 +40121,10 @@
         <v>0.219019</v>
       </c>
       <c r="D12" t="n">
-        <v>0.080931</v>
+        <v>0.122572</v>
       </c>
       <c r="E12" t="n">
-        <v>0.059084</v>
+        <v>0.089974</v>
       </c>
       <c r="F12" t="n">
         <v>0.1716417910447761</v>
@@ -40151,10 +40151,10 @@
         <v>0.43754</v>
       </c>
       <c r="D13" t="n">
-        <v>0.357774</v>
+        <v>0.280673</v>
       </c>
       <c r="E13" t="n">
-        <v>0.290111</v>
+        <v>0.226432</v>
       </c>
       <c r="F13" t="n">
         <v>0.3939393939393939</v>

</xml_diff>